<commit_message>
Actualizar derechos de autor
</commit_message>
<xml_diff>
--- a/data/diccionario_acuicultura.xlsx
+++ b/data/diccionario_acuicultura.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -379,7 +379,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>...1</t>
+          <t>TIPO_REG</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -388,7 +388,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>3447</v>
+        <v>1</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -397,7 +397,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TIPO_REG</t>
+          <t>PAIS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -415,7 +415,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PAIS</t>
+          <t>P_DEPTO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -433,7 +433,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P_DEPTO</t>
+          <t>P_MUNIC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -442,7 +442,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -451,7 +451,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P_MUNIC</t>
+          <t>UC_UO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -469,16 +469,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UC_UO</t>
+          <t>ENCUESTA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>character</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C7">
-        <v>662</v>
+        <v>2590</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -487,16 +487,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ENCUESTA</t>
+          <t>COD_VEREDA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>character</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C8">
-        <v>2590</v>
+        <v>870</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -505,7 +505,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COD_VEREDA</t>
+          <t>P_S7PNUMPEZ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -514,16 +514,16 @@
         </is>
       </c>
       <c r="C9">
-        <v>870</v>
+        <v>11</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P_S7PNUMPEZ</t>
+          <t>P_S7P96</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="C10">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -541,7 +541,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P_S7P96</t>
+          <t>P_S7P97</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -550,16 +550,16 @@
         </is>
       </c>
       <c r="C11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P_S7P97</t>
+          <t>P_S7P98</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="C12">
-        <v>13</v>
+        <v>125</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -577,7 +577,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P_S7P98</t>
+          <t>P_S7P99</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="C13">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -595,7 +595,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P_S7P99</t>
+          <t>P_S7P100</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -604,27 +604,9 @@
         </is>
       </c>
       <c r="C14">
-        <v>113</v>
+        <v>370</v>
       </c>
       <c r="D14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>P_S7P100</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="C15">
-        <v>370</v>
-      </c>
-      <c r="D15">
         <v>0</v>
       </c>
     </row>

</xml_diff>